<commit_message>
Add stress test HTML output, requirements, and updated scripts
</commit_message>
<xml_diff>
--- a/USAAA.xlsx
+++ b/USAAA.xlsx
@@ -1,80 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="Monthly" sheetId="2" r:id="rId2"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
-  <si>
-    <t>FRED Graph Observations</t>
-  </si>
-  <si>
-    <t>Federal Reserve Economic Data, Federal Reserve Bank of St. Louis</t>
-  </si>
-  <si>
-    <t>Link: https://fred.stlouisfed.org</t>
-  </si>
-  <si>
-    <t>Help: https://fredhelp.stlouisfed.org</t>
-  </si>
-  <si>
-    <t>This data may be copyrighted. Please refer to the Terms of Use: https://fred.stlouisfed.org/legal#fred-terms-faq</t>
-  </si>
-  <si>
-    <t>File Created: 2026-05-10 8:41 am CDT</t>
-  </si>
-  <si>
-    <t>DAAA</t>
-  </si>
-  <si>
-    <t>Moody's Seasoned Aaa Corporate Bond Yield, Percent, Monthly, Not Seasonally Adjusted</t>
-  </si>
-  <si>
-    <t>Data Updated: 2026-05-08</t>
-  </si>
-  <si>
-    <t>observation_date</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -107,22 +71,91 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -410,54 +443,76 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="85.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="79.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col width="85.7109375" customWidth="1" style="1" min="1" max="1"/>
+    <col width="79.140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="23.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FRED Graph Observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Federal Reserve Economic Data, Federal Reserve Bank of St. Louis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Link: https://fred.stlouisfed.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Help: https://fredhelp.stlouisfed.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>This data may be copyrighted. Please refer to the Terms of Use: https://fred.stlouisfed.org/legal#fred-terms-faq</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>File Created: 2026-05-10 8:41 am CDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>DAAA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Moody's Seasoned Aaa Corporate Bond Yield, Percent, Monthly, Not Seasonally Adjusted</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Data Updated: 2026-05-08</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -466,2036 +521,1948 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B253"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B241"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" style="2" bestFit="1" customWidth="1"/>
+    <col width="16.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="6.140625" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="4">
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>observation_date</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>DAAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
         <v>38353</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="5" t="n">
         <v>5.36</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="4">
+    <row r="3">
+      <c r="A3" s="6" t="n">
         <v>38384</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="5" t="n">
         <v>5.2</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="4">
+    <row r="4">
+      <c r="A4" s="6" t="n">
         <v>38412</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="5" t="n">
         <v>5.4</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="4">
+    <row r="5">
+      <c r="A5" s="6" t="n">
         <v>38443</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="5" t="n">
         <v>5.33</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="4">
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>38473</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="5" t="n">
         <v>5.15</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="4">
+    <row r="7">
+      <c r="A7" s="6" t="n">
         <v>38504</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="5" t="n">
         <v>4.96</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="4">
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>38534</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="5" t="n">
         <v>5.06</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="4">
+    <row r="9">
+      <c r="A9" s="6" t="n">
         <v>38565</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="5" t="n">
         <v>5.09</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="4">
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>38596</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="5" t="n">
         <v>5.13</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="4">
+    <row r="11">
+      <c r="A11" s="6" t="n">
         <v>38626</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="5" t="n">
         <v>5.35</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="4">
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>38657</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="5" t="n">
         <v>5.42</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="4">
+    <row r="13">
+      <c r="A13" s="6" t="n">
         <v>38687</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="5" t="n">
         <v>5.37</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="4">
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>38718</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="5" t="n">
         <v>5.29</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="4">
+    <row r="15">
+      <c r="A15" s="6" t="n">
         <v>38749</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="5" t="n">
         <v>5.35</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="4">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>38777</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="5" t="n">
         <v>5.53</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="4">
+    <row r="17">
+      <c r="A17" s="6" t="n">
         <v>38808</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="5" t="n">
         <v>5.84</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="4">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>38838</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="5" t="n">
         <v>5.95</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="4">
+    <row r="19">
+      <c r="A19" s="6" t="n">
         <v>38869</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="5" t="n">
         <v>5.89</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="4">
+    <row r="20">
+      <c r="A20" s="6" t="n">
         <v>38899</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="5" t="n">
         <v>5.85</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="4">
+    <row r="21">
+      <c r="A21" s="6" t="n">
         <v>38930</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="5" t="n">
         <v>5.68</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="4">
+    <row r="22">
+      <c r="A22" s="6" t="n">
         <v>38961</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="5" t="n">
         <v>5.51</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="4">
+    <row r="23">
+      <c r="A23" s="6" t="n">
         <v>38991</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="5" t="n">
         <v>5.51</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="4">
+    <row r="24">
+      <c r="A24" s="6" t="n">
         <v>39022</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="5" t="n">
         <v>5.33</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
-      <c r="A25" s="4">
+    <row r="25">
+      <c r="A25" s="6" t="n">
         <v>39052</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="5" t="n">
         <v>5.32</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="4">
+    <row r="26">
+      <c r="A26" s="6" t="n">
         <v>39083</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="5" t="n">
         <v>5.4</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
-      <c r="A27" s="4">
+    <row r="27">
+      <c r="A27" s="6" t="n">
         <v>39114</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="5" t="n">
         <v>5.39</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
-      <c r="A28" s="4">
+    <row r="28">
+      <c r="A28" s="6" t="n">
         <v>39142</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="5" t="n">
         <v>5.3</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
-      <c r="A29" s="4">
+    <row r="29">
+      <c r="A29" s="6" t="n">
         <v>39173</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="5" t="n">
         <v>5.47</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
-      <c r="A30" s="4">
+    <row r="30">
+      <c r="A30" s="6" t="n">
         <v>39203</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="5" t="n">
         <v>5.47</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
-      <c r="A31" s="4">
+    <row r="31">
+      <c r="A31" s="6" t="n">
         <v>39234</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="5" t="n">
         <v>5.79</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
-      <c r="A32" s="4">
+    <row r="32">
+      <c r="A32" s="6" t="n">
         <v>39264</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="5" t="n">
         <v>5.73</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
-      <c r="A33" s="4">
+    <row r="33">
+      <c r="A33" s="6" t="n">
         <v>39295</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="5" t="n">
         <v>5.79</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
-      <c r="A34" s="4">
+    <row r="34">
+      <c r="A34" s="6" t="n">
         <v>39326</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="5" t="n">
         <v>5.74</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
-      <c r="A35" s="4">
+    <row r="35">
+      <c r="A35" s="6" t="n">
         <v>39356</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="5" t="n">
         <v>5.66</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
-      <c r="A36" s="4">
+    <row r="36">
+      <c r="A36" s="6" t="n">
         <v>39387</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="5" t="n">
         <v>5.44</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
-      <c r="A37" s="4">
+    <row r="37">
+      <c r="A37" s="6" t="n">
         <v>39417</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="5" t="n">
         <v>5.49</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="4">
+    <row r="38">
+      <c r="A38" s="6" t="n">
         <v>39448</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="5" t="n">
         <v>5.33</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
-      <c r="A39" s="4">
+    <row r="39">
+      <c r="A39" s="6" t="n">
         <v>39479</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="5" t="n">
         <v>5.53</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="4">
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>39508</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="5" t="n">
         <v>5.51</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
-      <c r="A41" s="4">
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>39539</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="5" t="n">
         <v>5.55</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
-      <c r="A42" s="4">
+    <row r="42">
+      <c r="A42" s="6" t="n">
         <v>39569</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="5" t="n">
         <v>5.57</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
-      <c r="A43" s="4">
+    <row r="43">
+      <c r="A43" s="6" t="n">
         <v>39600</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="5" t="n">
         <v>5.68</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
-      <c r="A44" s="4">
+    <row r="44">
+      <c r="A44" s="6" t="n">
         <v>39630</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="5" t="n">
         <v>5.67</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
-      <c r="A45" s="4">
+    <row r="45">
+      <c r="A45" s="6" t="n">
         <v>39661</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="5" t="n">
         <v>5.64</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
-      <c r="A46" s="4">
+    <row r="46">
+      <c r="A46" s="6" t="n">
         <v>39692</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="5" t="n">
         <v>5.65</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
-      <c r="A47" s="4">
+    <row r="47">
+      <c r="A47" s="6" t="n">
         <v>39722</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="5" t="n">
         <v>6.28</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
-      <c r="A48" s="4">
+    <row r="48">
+      <c r="A48" s="6" t="n">
         <v>39753</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="5" t="n">
         <v>6.12</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
-      <c r="A49" s="4">
+    <row r="49">
+      <c r="A49" s="6" t="n">
         <v>39783</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="5" t="n">
         <v>5.05</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
-      <c r="A50" s="4">
+    <row r="50">
+      <c r="A50" s="6" t="n">
         <v>39814</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="5" t="n">
         <v>5.05</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
-      <c r="A51" s="4">
+    <row r="51">
+      <c r="A51" s="6" t="n">
         <v>39845</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="5" t="n">
         <v>5.27</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
-      <c r="A52" s="4">
+    <row r="52">
+      <c r="A52" s="6" t="n">
         <v>39873</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="5" t="n">
         <v>5.5</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
-      <c r="A53" s="4">
+    <row r="53">
+      <c r="A53" s="6" t="n">
         <v>39904</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="5" t="n">
         <v>5.39</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
-      <c r="A54" s="4">
+    <row r="54">
+      <c r="A54" s="6" t="n">
         <v>39934</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="5" t="n">
         <v>5.54</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
-      <c r="A55" s="4">
+    <row r="55">
+      <c r="A55" s="6" t="n">
         <v>39965</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="5" t="n">
         <v>5.61</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
-      <c r="A56" s="4">
+    <row r="56">
+      <c r="A56" s="6" t="n">
         <v>39995</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="5" t="n">
         <v>5.41</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
-      <c r="A57" s="4">
+    <row r="57">
+      <c r="A57" s="6" t="n">
         <v>40026</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="5" t="n">
         <v>5.26</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
-      <c r="A58" s="4">
+    <row r="58">
+      <c r="A58" s="6" t="n">
         <v>40057</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="5" t="n">
         <v>5.13</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
-      <c r="A59" s="4">
+    <row r="59">
+      <c r="A59" s="6" t="n">
         <v>40087</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="5" t="n">
         <v>5.15</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
-      <c r="A60" s="4">
+    <row r="60">
+      <c r="A60" s="6" t="n">
         <v>40118</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="5" t="n">
         <v>5.19</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
-      <c r="A61" s="4">
+    <row r="61">
+      <c r="A61" s="6" t="n">
         <v>40148</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="5" t="n">
         <v>5.26</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
-      <c r="A62" s="4">
+    <row r="62">
+      <c r="A62" s="6" t="n">
         <v>40179</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="5" t="n">
         <v>5.26</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
-      <c r="A63" s="4">
+    <row r="63">
+      <c r="A63" s="6" t="n">
         <v>40210</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="5" t="n">
         <v>5.35</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
-      <c r="A64" s="4">
+    <row r="64">
+      <c r="A64" s="6" t="n">
         <v>40238</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="5" t="n">
         <v>5.27</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
-      <c r="A65" s="4">
+    <row r="65">
+      <c r="A65" s="6" t="n">
         <v>40269</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="5" t="n">
         <v>5.29</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
-      <c r="A66" s="4">
+    <row r="66">
+      <c r="A66" s="6" t="n">
         <v>40299</v>
       </c>
-      <c r="B66" s="2">
+      <c r="B66" s="5" t="n">
         <v>4.96</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
-      <c r="A67" s="4">
+    <row r="67">
+      <c r="A67" s="6" t="n">
         <v>40330</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="5" t="n">
         <v>4.88</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
-      <c r="A68" s="4">
+    <row r="68">
+      <c r="A68" s="6" t="n">
         <v>40360</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="5" t="n">
         <v>4.72</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
-      <c r="A69" s="4">
+    <row r="69">
+      <c r="A69" s="6" t="n">
         <v>40391</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="5" t="n">
         <v>4.49</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
-      <c r="A70" s="4">
+    <row r="70">
+      <c r="A70" s="6" t="n">
         <v>40422</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="5" t="n">
         <v>4.53</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
-      <c r="A71" s="4">
+    <row r="71">
+      <c r="A71" s="6" t="n">
         <v>40452</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="5" t="n">
         <v>4.68</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
-      <c r="A72" s="4">
+    <row r="72">
+      <c r="A72" s="6" t="n">
         <v>40483</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="5" t="n">
         <v>4.87</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
-      <c r="A73" s="4">
+    <row r="73">
+      <c r="A73" s="6" t="n">
         <v>40513</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B73" s="5" t="n">
         <v>5.02</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
-      <c r="A74" s="4">
+    <row r="74">
+      <c r="A74" s="6" t="n">
         <v>40544</v>
       </c>
-      <c r="B74" s="2">
+      <c r="B74" s="5" t="n">
         <v>5.04</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
-      <c r="A75" s="4">
+    <row r="75">
+      <c r="A75" s="6" t="n">
         <v>40575</v>
       </c>
-      <c r="B75" s="2">
+      <c r="B75" s="5" t="n">
         <v>5.22</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="4">
+    <row r="76">
+      <c r="A76" s="6" t="n">
         <v>40603</v>
       </c>
-      <c r="B76" s="2">
+      <c r="B76" s="5" t="n">
         <v>5.13</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
-      <c r="A77" s="4">
+    <row r="77">
+      <c r="A77" s="6" t="n">
         <v>40634</v>
       </c>
-      <c r="B77" s="2">
+      <c r="B77" s="5" t="n">
         <v>5.16</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
-      <c r="A78" s="4">
+    <row r="78">
+      <c r="A78" s="6" t="n">
         <v>40664</v>
       </c>
-      <c r="B78" s="2">
+      <c r="B78" s="5" t="n">
         <v>4.96</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
-      <c r="A79" s="4">
+    <row r="79">
+      <c r="A79" s="6" t="n">
         <v>40695</v>
       </c>
-      <c r="B79" s="2">
+      <c r="B79" s="5" t="n">
         <v>4.99</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
-      <c r="A80" s="4">
+    <row r="80">
+      <c r="A80" s="6" t="n">
         <v>40725</v>
       </c>
-      <c r="B80" s="2">
+      <c r="B80" s="5" t="n">
         <v>4.93</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
-      <c r="A81" s="4">
+    <row r="81">
+      <c r="A81" s="6" t="n">
         <v>40756</v>
       </c>
-      <c r="B81" s="2">
+      <c r="B81" s="5" t="n">
         <v>4.37</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
-      <c r="A82" s="4">
+    <row r="82">
+      <c r="A82" s="6" t="n">
         <v>40787</v>
       </c>
-      <c r="B82" s="2">
+      <c r="B82" s="5" t="n">
         <v>4.09</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
-      <c r="A83" s="4">
+    <row r="83">
+      <c r="A83" s="6" t="n">
         <v>40817</v>
       </c>
-      <c r="B83" s="2">
+      <c r="B83" s="5" t="n">
         <v>3.98</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
-      <c r="A84" s="4">
+    <row r="84">
+      <c r="A84" s="6" t="n">
         <v>40848</v>
       </c>
-      <c r="B84" s="2">
+      <c r="B84" s="5" t="n">
         <v>3.87</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
-      <c r="A85" s="4">
+    <row r="85">
+      <c r="A85" s="6" t="n">
         <v>40878</v>
       </c>
-      <c r="B85" s="2">
+      <c r="B85" s="5" t="n">
         <v>3.93</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
-      <c r="A86" s="4">
+    <row r="86">
+      <c r="A86" s="6" t="n">
         <v>40909</v>
       </c>
-      <c r="B86" s="2">
+      <c r="B86" s="5" t="n">
         <v>3.85</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
-      <c r="A87" s="4">
+    <row r="87">
+      <c r="A87" s="6" t="n">
         <v>40940</v>
       </c>
-      <c r="B87" s="2">
+      <c r="B87" s="5" t="n">
         <v>3.85</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
-      <c r="A88" s="4">
+    <row r="88">
+      <c r="A88" s="6" t="n">
         <v>40969</v>
       </c>
-      <c r="B88" s="2">
+      <c r="B88" s="5" t="n">
         <v>3.99</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
-      <c r="A89" s="4">
+    <row r="89">
+      <c r="A89" s="6" t="n">
         <v>41000</v>
       </c>
-      <c r="B89" s="2">
+      <c r="B89" s="5" t="n">
         <v>3.96</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
-      <c r="A90" s="4">
+    <row r="90">
+      <c r="A90" s="6" t="n">
         <v>41030</v>
       </c>
-      <c r="B90" s="2">
+      <c r="B90" s="5" t="n">
         <v>3.8</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
-      <c r="A91" s="4">
+    <row r="91">
+      <c r="A91" s="6" t="n">
         <v>41061</v>
       </c>
-      <c r="B91" s="2">
+      <c r="B91" s="5" t="n">
         <v>3.64</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
-      <c r="A92" s="4">
+    <row r="92">
+      <c r="A92" s="6" t="n">
         <v>41091</v>
       </c>
-      <c r="B92" s="2">
+      <c r="B92" s="5" t="n">
         <v>3.4</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
-      <c r="A93" s="4">
+    <row r="93">
+      <c r="A93" s="6" t="n">
         <v>41122</v>
       </c>
-      <c r="B93" s="2">
+      <c r="B93" s="5" t="n">
         <v>3.48</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
-      <c r="A94" s="4">
+    <row r="94">
+      <c r="A94" s="6" t="n">
         <v>41153</v>
       </c>
-      <c r="B94" s="2">
+      <c r="B94" s="5" t="n">
         <v>3.49</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
-      <c r="A95" s="4">
+    <row r="95">
+      <c r="A95" s="6" t="n">
         <v>41183</v>
       </c>
-      <c r="B95" s="2">
+      <c r="B95" s="5" t="n">
         <v>3.47</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
-      <c r="A96" s="4">
+    <row r="96">
+      <c r="A96" s="6" t="n">
         <v>41214</v>
       </c>
-      <c r="B96" s="2">
+      <c r="B96" s="5" t="n">
         <v>3.5</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
-      <c r="A97" s="4">
+    <row r="97">
+      <c r="A97" s="6" t="n">
         <v>41244</v>
       </c>
-      <c r="B97" s="2">
+      <c r="B97" s="5" t="n">
         <v>3.65</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
-      <c r="A98" s="4">
+    <row r="98">
+      <c r="A98" s="6" t="n">
         <v>41275</v>
       </c>
-      <c r="B98" s="2">
+      <c r="B98" s="5" t="n">
         <v>3.8</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
-      <c r="A99" s="4">
+    <row r="99">
+      <c r="A99" s="6" t="n">
         <v>41306</v>
       </c>
-      <c r="B99" s="2">
+      <c r="B99" s="5" t="n">
         <v>3.9</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
-      <c r="A100" s="4">
+    <row r="100">
+      <c r="A100" s="6" t="n">
         <v>41334</v>
       </c>
-      <c r="B100" s="2">
+      <c r="B100" s="5" t="n">
         <v>3.93</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
-      <c r="A101" s="4">
+    <row r="101">
+      <c r="A101" s="6" t="n">
         <v>41365</v>
       </c>
-      <c r="B101" s="2">
+      <c r="B101" s="5" t="n">
         <v>3.73</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
-      <c r="A102" s="4">
+    <row r="102">
+      <c r="A102" s="6" t="n">
         <v>41395</v>
       </c>
-      <c r="B102" s="2">
+      <c r="B102" s="5" t="n">
         <v>3.89</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
-      <c r="A103" s="4">
+    <row r="103">
+      <c r="A103" s="6" t="n">
         <v>41426</v>
       </c>
-      <c r="B103" s="2">
+      <c r="B103" s="5" t="n">
         <v>4.27</v>
       </c>
     </row>
-    <row r="104" spans="1:2">
-      <c r="A104" s="4">
+    <row r="104">
+      <c r="A104" s="6" t="n">
         <v>41456</v>
       </c>
-      <c r="B104" s="2">
+      <c r="B104" s="5" t="n">
         <v>4.34</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
-      <c r="A105" s="4">
+    <row r="105">
+      <c r="A105" s="6" t="n">
         <v>41487</v>
       </c>
-      <c r="B105" s="2">
+      <c r="B105" s="5" t="n">
         <v>4.54</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
-      <c r="A106" s="4">
+    <row r="106">
+      <c r="A106" s="6" t="n">
         <v>41518</v>
       </c>
-      <c r="B106" s="2">
+      <c r="B106" s="5" t="n">
         <v>4.64</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
-      <c r="A107" s="4">
+    <row r="107">
+      <c r="A107" s="6" t="n">
         <v>41548</v>
       </c>
-      <c r="B107" s="2">
+      <c r="B107" s="5" t="n">
         <v>4.53</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
-      <c r="A108" s="4">
+    <row r="108">
+      <c r="A108" s="6" t="n">
         <v>41579</v>
       </c>
-      <c r="B108" s="2">
+      <c r="B108" s="5" t="n">
         <v>4.63</v>
       </c>
     </row>
-    <row r="109" spans="1:2">
-      <c r="A109" s="4">
+    <row r="109">
+      <c r="A109" s="6" t="n">
         <v>41609</v>
       </c>
-      <c r="B109" s="2">
+      <c r="B109" s="5" t="n">
         <v>4.62</v>
       </c>
     </row>
-    <row r="110" spans="1:2">
-      <c r="A110" s="4">
+    <row r="110">
+      <c r="A110" s="6" t="n">
         <v>41640</v>
       </c>
-      <c r="B110" s="2">
+      <c r="B110" s="5" t="n">
         <v>4.49</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
-      <c r="A111" s="4">
+    <row r="111">
+      <c r="A111" s="6" t="n">
         <v>41671</v>
       </c>
-      <c r="B111" s="2">
+      <c r="B111" s="5" t="n">
         <v>4.45</v>
       </c>
     </row>
-    <row r="112" spans="1:2">
-      <c r="A112" s="4">
+    <row r="112">
+      <c r="A112" s="6" t="n">
         <v>41699</v>
       </c>
-      <c r="B112" s="2">
+      <c r="B112" s="5" t="n">
         <v>4.38</v>
       </c>
     </row>
-    <row r="113" spans="1:2">
-      <c r="A113" s="4">
+    <row r="113">
+      <c r="A113" s="6" t="n">
         <v>41730</v>
       </c>
-      <c r="B113" s="2">
+      <c r="B113" s="5" t="n">
         <v>4.24</v>
       </c>
     </row>
-    <row r="114" spans="1:2">
-      <c r="A114" s="4">
+    <row r="114">
+      <c r="A114" s="6" t="n">
         <v>41760</v>
       </c>
-      <c r="B114" s="2">
+      <c r="B114" s="5" t="n">
         <v>4.16</v>
       </c>
     </row>
-    <row r="115" spans="1:2">
-      <c r="A115" s="4">
+    <row r="115">
+      <c r="A115" s="6" t="n">
         <v>41791</v>
       </c>
-      <c r="B115" s="2">
+      <c r="B115" s="5" t="n">
         <v>4.25</v>
       </c>
     </row>
-    <row r="116" spans="1:2">
-      <c r="A116" s="4">
+    <row r="116">
+      <c r="A116" s="6" t="n">
         <v>41821</v>
       </c>
-      <c r="B116" s="2">
+      <c r="B116" s="5" t="n">
         <v>4.16</v>
       </c>
     </row>
-    <row r="117" spans="1:2">
-      <c r="A117" s="4">
+    <row r="117">
+      <c r="A117" s="6" t="n">
         <v>41852</v>
       </c>
-      <c r="B117" s="2">
+      <c r="B117" s="5" t="n">
         <v>4.08</v>
       </c>
     </row>
-    <row r="118" spans="1:2">
-      <c r="A118" s="4">
+    <row r="118">
+      <c r="A118" s="6" t="n">
         <v>41883</v>
       </c>
-      <c r="B118" s="2">
+      <c r="B118" s="5" t="n">
         <v>4.11</v>
       </c>
     </row>
-    <row r="119" spans="1:2">
-      <c r="A119" s="4">
+    <row r="119">
+      <c r="A119" s="6" t="n">
         <v>41913</v>
       </c>
-      <c r="B119" s="2">
+      <c r="B119" s="5" t="n">
         <v>3.92</v>
       </c>
     </row>
-    <row r="120" spans="1:2">
-      <c r="A120" s="4">
+    <row r="120">
+      <c r="A120" s="6" t="n">
         <v>41944</v>
       </c>
-      <c r="B120" s="2">
+      <c r="B120" s="5" t="n">
         <v>3.92</v>
       </c>
     </row>
-    <row r="121" spans="1:2">
-      <c r="A121" s="4">
+    <row r="121">
+      <c r="A121" s="6" t="n">
         <v>41974</v>
       </c>
-      <c r="B121" s="2">
+      <c r="B121" s="5" t="n">
         <v>3.79</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
-      <c r="A122" s="4">
+    <row r="122">
+      <c r="A122" s="6" t="n">
         <v>42005</v>
       </c>
-      <c r="B122" s="2">
+      <c r="B122" s="5" t="n">
         <v>3.46</v>
       </c>
     </row>
-    <row r="123" spans="1:2">
-      <c r="A123" s="4">
+    <row r="123">
+      <c r="A123" s="6" t="n">
         <v>42036</v>
       </c>
-      <c r="B123" s="2">
+      <c r="B123" s="5" t="n">
         <v>3.61</v>
       </c>
     </row>
-    <row r="124" spans="1:2">
-      <c r="A124" s="4">
+    <row r="124">
+      <c r="A124" s="6" t="n">
         <v>42064</v>
       </c>
-      <c r="B124" s="2">
+      <c r="B124" s="5" t="n">
         <v>3.64</v>
       </c>
     </row>
-    <row r="125" spans="1:2">
-      <c r="A125" s="4">
+    <row r="125">
+      <c r="A125" s="6" t="n">
         <v>42095</v>
       </c>
-      <c r="B125" s="2">
+      <c r="B125" s="5" t="n">
         <v>3.52</v>
       </c>
     </row>
-    <row r="126" spans="1:2">
-      <c r="A126" s="4">
+    <row r="126">
+      <c r="A126" s="6" t="n">
         <v>42125</v>
       </c>
-      <c r="B126" s="2">
+      <c r="B126" s="5" t="n">
         <v>3.98</v>
       </c>
     </row>
-    <row r="127" spans="1:2">
-      <c r="A127" s="4">
+    <row r="127">
+      <c r="A127" s="6" t="n">
         <v>42156</v>
       </c>
-      <c r="B127" s="2">
+      <c r="B127" s="5" t="n">
         <v>4.19</v>
       </c>
     </row>
-    <row r="128" spans="1:2">
-      <c r="A128" s="4">
+    <row r="128">
+      <c r="A128" s="6" t="n">
         <v>42186</v>
       </c>
-      <c r="B128" s="2">
+      <c r="B128" s="5" t="n">
         <v>4.15</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
-      <c r="A129" s="4">
+    <row r="129">
+      <c r="A129" s="6" t="n">
         <v>42217</v>
       </c>
-      <c r="B129" s="2">
+      <c r="B129" s="5" t="n">
         <v>4.04</v>
       </c>
     </row>
-    <row r="130" spans="1:2">
-      <c r="A130" s="4">
+    <row r="130">
+      <c r="A130" s="6" t="n">
         <v>42248</v>
       </c>
-      <c r="B130" s="2">
+      <c r="B130" s="5" t="n">
         <v>4.07</v>
       </c>
     </row>
-    <row r="131" spans="1:2">
-      <c r="A131" s="4">
+    <row r="131">
+      <c r="A131" s="6" t="n">
         <v>42278</v>
       </c>
-      <c r="B131" s="2">
+      <c r="B131" s="5" t="n">
         <v>3.95</v>
       </c>
     </row>
-    <row r="132" spans="1:2">
-      <c r="A132" s="4">
+    <row r="132">
+      <c r="A132" s="6" t="n">
         <v>42309</v>
       </c>
-      <c r="B132" s="2">
+      <c r="B132" s="5" t="n">
         <v>4.06</v>
       </c>
     </row>
-    <row r="133" spans="1:2">
-      <c r="A133" s="4">
+    <row r="133">
+      <c r="A133" s="6" t="n">
         <v>42339</v>
       </c>
-      <c r="B133" s="2">
+      <c r="B133" s="5" t="n">
         <v>3.97</v>
       </c>
     </row>
-    <row r="134" spans="1:2">
-      <c r="A134" s="4">
+    <row r="134">
+      <c r="A134" s="6" t="n">
         <v>42370</v>
       </c>
-      <c r="B134" s="2">
+      <c r="B134" s="5" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:2">
-      <c r="A135" s="4">
+    <row r="135">
+      <c r="A135" s="6" t="n">
         <v>42401</v>
       </c>
-      <c r="B135" s="2">
+      <c r="B135" s="5" t="n">
         <v>3.96</v>
       </c>
     </row>
-    <row r="136" spans="1:2">
-      <c r="A136" s="4">
+    <row r="136">
+      <c r="A136" s="6" t="n">
         <v>42430</v>
       </c>
-      <c r="B136" s="2">
+      <c r="B136" s="5" t="n">
         <v>3.82</v>
       </c>
     </row>
-    <row r="137" spans="1:2">
-      <c r="A137" s="4">
+    <row r="137">
+      <c r="A137" s="6" t="n">
         <v>42461</v>
       </c>
-      <c r="B137" s="2">
+      <c r="B137" s="5" t="n">
         <v>3.62</v>
       </c>
     </row>
-    <row r="138" spans="1:2">
-      <c r="A138" s="4">
+    <row r="138">
+      <c r="A138" s="6" t="n">
         <v>42491</v>
       </c>
-      <c r="B138" s="2">
+      <c r="B138" s="5" t="n">
         <v>3.65</v>
       </c>
     </row>
-    <row r="139" spans="1:2">
-      <c r="A139" s="4">
+    <row r="139">
+      <c r="A139" s="6" t="n">
         <v>42522</v>
       </c>
-      <c r="B139" s="2">
+      <c r="B139" s="5" t="n">
         <v>3.5</v>
       </c>
     </row>
-    <row r="140" spans="1:2">
-      <c r="A140" s="4">
+    <row r="140">
+      <c r="A140" s="6" t="n">
         <v>42552</v>
       </c>
-      <c r="B140" s="2">
+      <c r="B140" s="5" t="n">
         <v>3.28</v>
       </c>
     </row>
-    <row r="141" spans="1:2">
-      <c r="A141" s="4">
+    <row r="141">
+      <c r="A141" s="6" t="n">
         <v>42583</v>
       </c>
-      <c r="B141" s="2">
+      <c r="B141" s="5" t="n">
         <v>3.32</v>
       </c>
     </row>
-    <row r="142" spans="1:2">
-      <c r="A142" s="4">
+    <row r="142">
+      <c r="A142" s="6" t="n">
         <v>42614</v>
       </c>
-      <c r="B142" s="2">
+      <c r="B142" s="5" t="n">
         <v>3.41</v>
       </c>
     </row>
-    <row r="143" spans="1:2">
-      <c r="A143" s="4">
+    <row r="143">
+      <c r="A143" s="6" t="n">
         <v>42644</v>
       </c>
-      <c r="B143" s="2">
+      <c r="B143" s="5" t="n">
         <v>3.51</v>
       </c>
     </row>
-    <row r="144" spans="1:2">
-      <c r="A144" s="4">
+    <row r="144">
+      <c r="A144" s="6" t="n">
         <v>42675</v>
       </c>
-      <c r="B144" s="2">
+      <c r="B144" s="5" t="n">
         <v>3.86</v>
       </c>
     </row>
-    <row r="145" spans="1:2">
-      <c r="A145" s="4">
+    <row r="145">
+      <c r="A145" s="6" t="n">
         <v>42705</v>
       </c>
-      <c r="B145" s="2">
+      <c r="B145" s="5" t="n">
         <v>4.06</v>
       </c>
     </row>
-    <row r="146" spans="1:2">
-      <c r="A146" s="4">
+    <row r="146">
+      <c r="A146" s="6" t="n">
         <v>42736</v>
       </c>
-      <c r="B146" s="2">
+      <c r="B146" s="5" t="n">
         <v>3.92</v>
       </c>
     </row>
-    <row r="147" spans="1:2">
-      <c r="A147" s="4">
+    <row r="147">
+      <c r="A147" s="6" t="n">
         <v>42767</v>
       </c>
-      <c r="B147" s="2">
+      <c r="B147" s="5" t="n">
         <v>3.95</v>
       </c>
     </row>
-    <row r="148" spans="1:2">
-      <c r="A148" s="4">
+    <row r="148">
+      <c r="A148" s="6" t="n">
         <v>42795</v>
       </c>
-      <c r="B148" s="2">
+      <c r="B148" s="5" t="n">
         <v>4.01</v>
       </c>
     </row>
-    <row r="149" spans="1:2">
-      <c r="A149" s="4">
+    <row r="149">
+      <c r="A149" s="6" t="n">
         <v>42826</v>
       </c>
-      <c r="B149" s="2">
+      <c r="B149" s="5" t="n">
         <v>3.87</v>
       </c>
     </row>
-    <row r="150" spans="1:2">
-      <c r="A150" s="4">
+    <row r="150">
+      <c r="A150" s="6" t="n">
         <v>42856</v>
       </c>
-      <c r="B150" s="2">
+      <c r="B150" s="5" t="n">
         <v>3.85</v>
       </c>
     </row>
-    <row r="151" spans="1:2">
-      <c r="A151" s="4">
+    <row r="151">
+      <c r="A151" s="6" t="n">
         <v>42887</v>
       </c>
-      <c r="B151" s="2">
+      <c r="B151" s="5" t="n">
         <v>3.68</v>
       </c>
     </row>
-    <row r="152" spans="1:2">
-      <c r="A152" s="4">
+    <row r="152">
+      <c r="A152" s="6" t="n">
         <v>42917</v>
       </c>
-      <c r="B152" s="2">
+      <c r="B152" s="5" t="n">
         <v>3.7</v>
       </c>
     </row>
-    <row r="153" spans="1:2">
-      <c r="A153" s="4">
+    <row r="153">
+      <c r="A153" s="6" t="n">
         <v>42948</v>
       </c>
-      <c r="B153" s="2">
+      <c r="B153" s="5" t="n">
         <v>3.63</v>
       </c>
     </row>
-    <row r="154" spans="1:2">
-      <c r="A154" s="4">
+    <row r="154">
+      <c r="A154" s="6" t="n">
         <v>42979</v>
       </c>
-      <c r="B154" s="2">
+      <c r="B154" s="5" t="n">
         <v>3.63</v>
       </c>
     </row>
-    <row r="155" spans="1:2">
-      <c r="A155" s="4">
+    <row r="155">
+      <c r="A155" s="6" t="n">
         <v>43009</v>
       </c>
-      <c r="B155" s="2">
+      <c r="B155" s="5" t="n">
         <v>3.6</v>
       </c>
     </row>
-    <row r="156" spans="1:2">
-      <c r="A156" s="4">
+    <row r="156">
+      <c r="A156" s="6" t="n">
         <v>43040</v>
       </c>
-      <c r="B156" s="2">
+      <c r="B156" s="5" t="n">
         <v>3.57</v>
       </c>
     </row>
-    <row r="157" spans="1:2">
-      <c r="A157" s="4">
+    <row r="157">
+      <c r="A157" s="6" t="n">
         <v>43070</v>
       </c>
-      <c r="B157" s="2">
+      <c r="B157" s="5" t="n">
         <v>3.51</v>
       </c>
     </row>
-    <row r="158" spans="1:2">
-      <c r="A158" s="4">
+    <row r="158">
+      <c r="A158" s="6" t="n">
         <v>43101</v>
       </c>
-      <c r="B158" s="2">
+      <c r="B158" s="5" t="n">
         <v>3.55</v>
       </c>
     </row>
-    <row r="159" spans="1:2">
-      <c r="A159" s="4">
+    <row r="159">
+      <c r="A159" s="6" t="n">
         <v>43132</v>
       </c>
-      <c r="B159" s="2">
+      <c r="B159" s="5" t="n">
         <v>3.82</v>
       </c>
     </row>
-    <row r="160" spans="1:2">
-      <c r="A160" s="4">
+    <row r="160">
+      <c r="A160" s="6" t="n">
         <v>43160</v>
       </c>
-      <c r="B160" s="2">
+      <c r="B160" s="5" t="n">
         <v>3.87</v>
       </c>
     </row>
-    <row r="161" spans="1:2">
-      <c r="A161" s="4">
+    <row r="161">
+      <c r="A161" s="6" t="n">
         <v>43191</v>
       </c>
-      <c r="B161" s="2">
+      <c r="B161" s="5" t="n">
         <v>3.85</v>
       </c>
     </row>
-    <row r="162" spans="1:2">
-      <c r="A162" s="4">
+    <row r="162">
+      <c r="A162" s="6" t="n">
         <v>43221</v>
       </c>
-      <c r="B162" s="2">
+      <c r="B162" s="5" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="163" spans="1:2">
-      <c r="A163" s="4">
+    <row r="163">
+      <c r="A163" s="6" t="n">
         <v>43252</v>
       </c>
-      <c r="B163" s="2">
+      <c r="B163" s="5" t="n">
         <v>3.96</v>
       </c>
     </row>
-    <row r="164" spans="1:2">
-      <c r="A164" s="4">
+    <row r="164">
+      <c r="A164" s="6" t="n">
         <v>43282</v>
       </c>
-      <c r="B164" s="2">
+      <c r="B164" s="5" t="n">
         <v>3.87</v>
       </c>
     </row>
-    <row r="165" spans="1:2">
-      <c r="A165" s="4">
+    <row r="165">
+      <c r="A165" s="6" t="n">
         <v>43313</v>
       </c>
-      <c r="B165" s="2">
+      <c r="B165" s="5" t="n">
         <v>3.88</v>
       </c>
     </row>
-    <row r="166" spans="1:2">
-      <c r="A166" s="4">
+    <row r="166">
+      <c r="A166" s="6" t="n">
         <v>43344</v>
       </c>
-      <c r="B166" s="2">
+      <c r="B166" s="5" t="n">
         <v>3.98</v>
       </c>
     </row>
-    <row r="167" spans="1:2">
-      <c r="A167" s="4">
+    <row r="167">
+      <c r="A167" s="6" t="n">
         <v>43374</v>
       </c>
-      <c r="B167" s="2">
+      <c r="B167" s="5" t="n">
         <v>4.14</v>
       </c>
     </row>
-    <row r="168" spans="1:2">
-      <c r="A168" s="4">
+    <row r="168">
+      <c r="A168" s="6" t="n">
         <v>43405</v>
       </c>
-      <c r="B168" s="2">
+      <c r="B168" s="5" t="n">
         <v>4.22</v>
       </c>
     </row>
-    <row r="169" spans="1:2">
-      <c r="A169" s="4">
+    <row r="169">
+      <c r="A169" s="6" t="n">
         <v>43435</v>
       </c>
-      <c r="B169" s="2">
+      <c r="B169" s="5" t="n">
         <v>4.02</v>
       </c>
     </row>
-    <row r="170" spans="1:2">
-      <c r="A170" s="4">
+    <row r="170">
+      <c r="A170" s="6" t="n">
         <v>43466</v>
       </c>
-      <c r="B170" s="2">
+      <c r="B170" s="5" t="n">
         <v>3.93</v>
       </c>
     </row>
-    <row r="171" spans="1:2">
-      <c r="A171" s="4">
+    <row r="171">
+      <c r="A171" s="6" t="n">
         <v>43497</v>
       </c>
-      <c r="B171" s="2">
+      <c r="B171" s="5" t="n">
         <v>3.79</v>
       </c>
     </row>
-    <row r="172" spans="1:2">
-      <c r="A172" s="4">
+    <row r="172">
+      <c r="A172" s="6" t="n">
         <v>43525</v>
       </c>
-      <c r="B172" s="2">
+      <c r="B172" s="5" t="n">
         <v>3.77</v>
       </c>
     </row>
-    <row r="173" spans="1:2">
-      <c r="A173" s="4">
+    <row r="173">
+      <c r="A173" s="6" t="n">
         <v>43556</v>
       </c>
-      <c r="B173" s="2">
+      <c r="B173" s="5" t="n">
         <v>3.69</v>
       </c>
     </row>
-    <row r="174" spans="1:2">
-      <c r="A174" s="4">
+    <row r="174">
+      <c r="A174" s="6" t="n">
         <v>43586</v>
       </c>
-      <c r="B174" s="2">
+      <c r="B174" s="5" t="n">
         <v>3.67</v>
       </c>
     </row>
-    <row r="175" spans="1:2">
-      <c r="A175" s="4">
+    <row r="175">
+      <c r="A175" s="6" t="n">
         <v>43617</v>
       </c>
-      <c r="B175" s="2">
+      <c r="B175" s="5" t="n">
         <v>3.42</v>
       </c>
     </row>
-    <row r="176" spans="1:2">
-      <c r="A176" s="4">
+    <row r="176">
+      <c r="A176" s="6" t="n">
         <v>43647</v>
       </c>
-      <c r="B176" s="2">
+      <c r="B176" s="5" t="n">
         <v>3.29</v>
       </c>
     </row>
-    <row r="177" spans="1:2">
-      <c r="A177" s="4">
+    <row r="177">
+      <c r="A177" s="6" t="n">
         <v>43678</v>
       </c>
-      <c r="B177" s="2">
+      <c r="B177" s="5" t="n">
         <v>2.98</v>
       </c>
     </row>
-    <row r="178" spans="1:2">
-      <c r="A178" s="4">
+    <row r="178">
+      <c r="A178" s="6" t="n">
         <v>43709</v>
       </c>
-      <c r="B178" s="2">
+      <c r="B178" s="5" t="n">
         <v>3.03</v>
       </c>
     </row>
-    <row r="179" spans="1:2">
-      <c r="A179" s="4">
+    <row r="179">
+      <c r="A179" s="6" t="n">
         <v>43739</v>
       </c>
-      <c r="B179" s="2">
+      <c r="B179" s="5" t="n">
         <v>3.01</v>
       </c>
     </row>
-    <row r="180" spans="1:2">
-      <c r="A180" s="4">
+    <row r="180">
+      <c r="A180" s="6" t="n">
         <v>43770</v>
       </c>
-      <c r="B180" s="2">
+      <c r="B180" s="5" t="n">
         <v>3.06</v>
       </c>
     </row>
-    <row r="181" spans="1:2">
-      <c r="A181" s="4">
+    <row r="181">
+      <c r="A181" s="6" t="n">
         <v>43800</v>
       </c>
-      <c r="B181" s="2">
+      <c r="B181" s="5" t="n">
         <v>3.01</v>
       </c>
     </row>
-    <row r="182" spans="1:2">
-      <c r="A182" s="4">
+    <row r="182">
+      <c r="A182" s="6" t="n">
         <v>43831</v>
       </c>
-      <c r="B182" s="2">
+      <c r="B182" s="5" t="n">
         <v>2.94</v>
       </c>
     </row>
-    <row r="183" spans="1:2">
-      <c r="A183" s="4">
+    <row r="183">
+      <c r="A183" s="6" t="n">
         <v>43862</v>
       </c>
-      <c r="B183" s="2">
+      <c r="B183" s="5" t="n">
         <v>2.78</v>
       </c>
     </row>
-    <row r="184" spans="1:2">
-      <c r="A184" s="4">
+    <row r="184">
+      <c r="A184" s="6" t="n">
         <v>43891</v>
       </c>
-      <c r="B184" s="2">
+      <c r="B184" s="5" t="n">
         <v>3.02</v>
       </c>
     </row>
-    <row r="185" spans="1:2">
-      <c r="A185" s="4">
+    <row r="185">
+      <c r="A185" s="6" t="n">
         <v>43922</v>
       </c>
-      <c r="B185" s="2">
+      <c r="B185" s="5" t="n">
         <v>2.43</v>
       </c>
     </row>
-    <row r="186" spans="1:2">
-      <c r="A186" s="4">
+    <row r="186">
+      <c r="A186" s="6" t="n">
         <v>43952</v>
       </c>
-      <c r="B186" s="2">
+      <c r="B186" s="5" t="n">
         <v>2.5</v>
       </c>
     </row>
-    <row r="187" spans="1:2">
-      <c r="A187" s="4">
+    <row r="187">
+      <c r="A187" s="6" t="n">
         <v>43983</v>
       </c>
-      <c r="B187" s="2">
+      <c r="B187" s="5" t="n">
         <v>2.44</v>
       </c>
     </row>
-    <row r="188" spans="1:2">
-      <c r="A188" s="4">
+    <row r="188">
+      <c r="A188" s="6" t="n">
         <v>44013</v>
       </c>
-      <c r="B188" s="2">
+      <c r="B188" s="5" t="n">
         <v>2.14</v>
       </c>
     </row>
-    <row r="189" spans="1:2">
-      <c r="A189" s="4">
+    <row r="189">
+      <c r="A189" s="6" t="n">
         <v>44044</v>
       </c>
-      <c r="B189" s="2">
+      <c r="B189" s="5" t="n">
         <v>2.25</v>
       </c>
     </row>
-    <row r="190" spans="1:2">
-      <c r="A190" s="4">
+    <row r="190">
+      <c r="A190" s="6" t="n">
         <v>44075</v>
       </c>
-      <c r="B190" s="2">
+      <c r="B190" s="5" t="n">
         <v>2.31</v>
       </c>
     </row>
-    <row r="191" spans="1:2">
-      <c r="A191" s="4">
+    <row r="191">
+      <c r="A191" s="6" t="n">
         <v>44105</v>
       </c>
-      <c r="B191" s="2">
+      <c r="B191" s="5" t="n">
         <v>2.35</v>
       </c>
     </row>
-    <row r="192" spans="1:2">
-      <c r="A192" s="4">
+    <row r="192">
+      <c r="A192" s="6" t="n">
         <v>44136</v>
       </c>
-      <c r="B192" s="2">
+      <c r="B192" s="5" t="n">
         <v>2.3</v>
       </c>
     </row>
-    <row r="193" spans="1:2">
-      <c r="A193" s="4">
+    <row r="193">
+      <c r="A193" s="6" t="n">
         <v>44166</v>
       </c>
-      <c r="B193" s="2">
+      <c r="B193" s="5" t="n">
         <v>2.26</v>
       </c>
     </row>
-    <row r="194" spans="1:2">
-      <c r="A194" s="4">
+    <row r="194">
+      <c r="A194" s="6" t="n">
         <v>44197</v>
       </c>
-      <c r="B194" s="2">
+      <c r="B194" s="5" t="n">
         <v>2.45</v>
       </c>
     </row>
-    <row r="195" spans="1:2">
-      <c r="A195" s="4">
+    <row r="195">
+      <c r="A195" s="6" t="n">
         <v>44228</v>
       </c>
-      <c r="B195" s="2">
+      <c r="B195" s="5" t="n">
         <v>2.7</v>
       </c>
     </row>
-    <row r="196" spans="1:2">
-      <c r="A196" s="4">
+    <row r="196">
+      <c r="A196" s="6" t="n">
         <v>44256</v>
       </c>
-      <c r="B196" s="2">
+      <c r="B196" s="5" t="n">
         <v>3.04</v>
       </c>
     </row>
-    <row r="197" spans="1:2">
-      <c r="A197" s="4">
+    <row r="197">
+      <c r="A197" s="6" t="n">
         <v>44287</v>
       </c>
-      <c r="B197" s="2">
+      <c r="B197" s="5" t="n">
         <v>2.9</v>
       </c>
     </row>
-    <row r="198" spans="1:2">
-      <c r="A198" s="4">
+    <row r="198">
+      <c r="A198" s="6" t="n">
         <v>44317</v>
       </c>
-      <c r="B198" s="2">
+      <c r="B198" s="5" t="n">
         <v>2.96</v>
       </c>
     </row>
-    <row r="199" spans="1:2">
-      <c r="A199" s="4">
+    <row r="199">
+      <c r="A199" s="6" t="n">
         <v>44348</v>
       </c>
-      <c r="B199" s="2">
+      <c r="B199" s="5" t="n">
         <v>2.79</v>
       </c>
     </row>
-    <row r="200" spans="1:2">
-      <c r="A200" s="4">
+    <row r="200">
+      <c r="A200" s="6" t="n">
         <v>44378</v>
       </c>
-      <c r="B200" s="2">
+      <c r="B200" s="5" t="n">
         <v>2.57</v>
       </c>
     </row>
-    <row r="201" spans="1:2">
-      <c r="A201" s="4">
+    <row r="201">
+      <c r="A201" s="6" t="n">
         <v>44409</v>
       </c>
-      <c r="B201" s="2">
+      <c r="B201" s="5" t="n">
         <v>2.55</v>
       </c>
     </row>
-    <row r="202" spans="1:2">
-      <c r="A202" s="4">
+    <row r="202">
+      <c r="A202" s="6" t="n">
         <v>44440</v>
       </c>
-      <c r="B202" s="2">
+      <c r="B202" s="5" t="n">
         <v>2.53</v>
       </c>
     </row>
-    <row r="203" spans="1:2">
-      <c r="A203" s="4">
+    <row r="203">
+      <c r="A203" s="6" t="n">
         <v>44470</v>
       </c>
-      <c r="B203" s="2">
+      <c r="B203" s="5" t="n">
         <v>2.68</v>
       </c>
     </row>
-    <row r="204" spans="1:2">
-      <c r="A204" s="4">
+    <row r="204">
+      <c r="A204" s="6" t="n">
         <v>44501</v>
       </c>
-      <c r="B204" s="2">
+      <c r="B204" s="5" t="n">
         <v>2.62</v>
       </c>
     </row>
-    <row r="205" spans="1:2">
-      <c r="A205" s="4">
+    <row r="205">
+      <c r="A205" s="6" t="n">
         <v>44531</v>
       </c>
-      <c r="B205" s="2">
+      <c r="B205" s="5" t="n">
         <v>2.64</v>
       </c>
     </row>
-    <row r="206" spans="1:2">
-      <c r="A206" s="4">
+    <row r="206">
+      <c r="A206" s="6" t="n">
         <v>44562</v>
       </c>
-      <c r="B206" s="2">
+      <c r="B206" s="5" t="n">
         <v>2.93</v>
       </c>
     </row>
-    <row r="207" spans="1:2">
-      <c r="A207" s="4">
+    <row r="207">
+      <c r="A207" s="6" t="n">
         <v>44593</v>
       </c>
-      <c r="B207" s="2">
+      <c r="B207" s="5" t="n">
         <v>3.25</v>
       </c>
     </row>
-    <row r="208" spans="1:2">
-      <c r="A208" s="4">
+    <row r="208">
+      <c r="A208" s="6" t="n">
         <v>44621</v>
       </c>
-      <c r="B208" s="2">
+      <c r="B208" s="5" t="n">
         <v>3.43</v>
       </c>
     </row>
-    <row r="209" spans="1:2">
-      <c r="A209" s="4">
+    <row r="209">
+      <c r="A209" s="6" t="n">
         <v>44652</v>
       </c>
-      <c r="B209" s="2">
+      <c r="B209" s="5" t="n">
         <v>3.76</v>
       </c>
     </row>
-    <row r="210" spans="1:2">
-      <c r="A210" s="4">
+    <row r="210">
+      <c r="A210" s="6" t="n">
         <v>44682</v>
       </c>
-      <c r="B210" s="2">
+      <c r="B210" s="5" t="n">
         <v>4.13</v>
       </c>
     </row>
-    <row r="211" spans="1:2">
-      <c r="A211" s="4">
+    <row r="211">
+      <c r="A211" s="6" t="n">
         <v>44713</v>
       </c>
-      <c r="B211" s="2">
+      <c r="B211" s="5" t="n">
         <v>4.24</v>
       </c>
     </row>
-    <row r="212" spans="1:2">
-      <c r="A212" s="4">
+    <row r="212">
+      <c r="A212" s="6" t="n">
         <v>44743</v>
       </c>
-      <c r="B212" s="2">
+      <c r="B212" s="5" t="n">
         <v>4.06</v>
       </c>
     </row>
-    <row r="213" spans="1:2">
-      <c r="A213" s="4">
+    <row r="213">
+      <c r="A213" s="6" t="n">
         <v>44774</v>
       </c>
-      <c r="B213" s="2">
+      <c r="B213" s="5" t="n">
         <v>4.07</v>
       </c>
     </row>
-    <row r="214" spans="1:2">
-      <c r="A214" s="4">
+    <row r="214">
+      <c r="A214" s="6" t="n">
         <v>44805</v>
       </c>
-      <c r="B214" s="2">
+      <c r="B214" s="5" t="n">
         <v>4.59</v>
       </c>
     </row>
-    <row r="215" spans="1:2">
-      <c r="A215" s="4">
+    <row r="215">
+      <c r="A215" s="6" t="n">
         <v>44835</v>
       </c>
-      <c r="B215" s="2">
+      <c r="B215" s="5" t="n">
         <v>5.1</v>
       </c>
     </row>
-    <row r="216" spans="1:2">
-      <c r="A216" s="4">
+    <row r="216">
+      <c r="A216" s="6" t="n">
         <v>44866</v>
       </c>
-      <c r="B216" s="2">
+      <c r="B216" s="5" t="n">
         <v>4.9</v>
       </c>
     </row>
-    <row r="217" spans="1:2">
-      <c r="A217" s="4">
+    <row r="217">
+      <c r="A217" s="6" t="n">
         <v>44896</v>
       </c>
-      <c r="B217" s="2">
+      <c r="B217" s="5" t="n">
         <v>4.43</v>
       </c>
     </row>
-    <row r="218" spans="1:2">
-      <c r="A218" s="4">
+    <row r="218">
+      <c r="A218" s="6" t="n">
         <v>44927</v>
       </c>
-      <c r="B218" s="2">
+      <c r="B218" s="5" t="n">
         <v>4.4</v>
       </c>
     </row>
-    <row r="219" spans="1:2">
-      <c r="A219" s="4">
+    <row r="219">
+      <c r="A219" s="6" t="n">
         <v>44958</v>
       </c>
-      <c r="B219" s="2">
+      <c r="B219" s="5" t="n">
         <v>4.56</v>
       </c>
     </row>
-    <row r="220" spans="1:2">
-      <c r="A220" s="4">
+    <row r="220">
+      <c r="A220" s="6" t="n">
         <v>44986</v>
       </c>
-      <c r="B220" s="2">
+      <c r="B220" s="5" t="n">
         <v>4.6</v>
       </c>
     </row>
-    <row r="221" spans="1:2">
-      <c r="A221" s="4">
+    <row r="221">
+      <c r="A221" s="6" t="n">
         <v>45017</v>
       </c>
-      <c r="B221" s="2">
+      <c r="B221" s="5" t="n">
         <v>4.47</v>
       </c>
     </row>
-    <row r="222" spans="1:2">
-      <c r="A222" s="4">
+    <row r="222">
+      <c r="A222" s="6" t="n">
         <v>45047</v>
       </c>
-      <c r="B222" s="2">
+      <c r="B222" s="5" t="n">
         <v>4.67</v>
       </c>
     </row>
-    <row r="223" spans="1:2">
-      <c r="A223" s="4">
+    <row r="223">
+      <c r="A223" s="6" t="n">
         <v>45078</v>
       </c>
-      <c r="B223" s="2">
+      <c r="B223" s="5" t="n">
         <v>4.65</v>
       </c>
     </row>
-    <row r="224" spans="1:2">
-      <c r="A224" s="4">
+    <row r="224">
+      <c r="A224" s="6" t="n">
         <v>45108</v>
       </c>
-      <c r="B224" s="2">
+      <c r="B224" s="5" t="n">
         <v>4.66</v>
       </c>
     </row>
-    <row r="225" spans="1:2">
-      <c r="A225" s="4">
+    <row r="225">
+      <c r="A225" s="6" t="n">
         <v>45139</v>
       </c>
-      <c r="B225" s="2">
+      <c r="B225" s="5" t="n">
         <v>4.95</v>
       </c>
     </row>
-    <row r="226" spans="1:2">
-      <c r="A226" s="4">
+    <row r="226">
+      <c r="A226" s="6" t="n">
         <v>45170</v>
       </c>
-      <c r="B226" s="2">
+      <c r="B226" s="5" t="n">
         <v>5.13</v>
       </c>
     </row>
-    <row r="227" spans="1:2">
-      <c r="A227" s="4">
+    <row r="227">
+      <c r="A227" s="6" t="n">
         <v>45200</v>
       </c>
-      <c r="B227" s="2">
+      <c r="B227" s="5" t="n">
         <v>5.61</v>
       </c>
     </row>
-    <row r="228" spans="1:2">
-      <c r="A228" s="4">
+    <row r="228">
+      <c r="A228" s="6" t="n">
         <v>45231</v>
       </c>
-      <c r="B228" s="2">
+      <c r="B228" s="5" t="n">
         <v>5.28</v>
       </c>
     </row>
-    <row r="229" spans="1:2">
-      <c r="A229" s="4">
+    <row r="229">
+      <c r="A229" s="6" t="n">
         <v>45261</v>
       </c>
-      <c r="B229" s="2">
+      <c r="B229" s="5" t="n">
         <v>4.74</v>
       </c>
     </row>
-    <row r="230" spans="1:2">
-      <c r="A230" s="4">
+    <row r="230">
+      <c r="A230" s="6" t="n">
         <v>45292</v>
       </c>
-      <c r="B230" s="2">
+      <c r="B230" s="5" t="n">
         <v>4.87</v>
       </c>
     </row>
-    <row r="231" spans="1:2">
-      <c r="A231" s="4">
+    <row r="231">
+      <c r="A231" s="6" t="n">
         <v>45323</v>
       </c>
-      <c r="B231" s="2">
+      <c r="B231" s="5" t="n">
         <v>5.03</v>
       </c>
     </row>
-    <row r="232" spans="1:2">
-      <c r="A232" s="4">
+    <row r="232">
+      <c r="A232" s="6" t="n">
         <v>45352</v>
       </c>
-      <c r="B232" s="2">
+      <c r="B232" s="5" t="n">
         <v>5.01</v>
       </c>
     </row>
-    <row r="233" spans="1:2">
-      <c r="A233" s="4">
+    <row r="233">
+      <c r="A233" s="6" t="n">
         <v>45383</v>
       </c>
-      <c r="B233" s="2">
+      <c r="B233" s="5" t="n">
         <v>5.28</v>
       </c>
     </row>
-    <row r="234" spans="1:2">
-      <c r="A234" s="4">
+    <row r="234">
+      <c r="A234" s="6" t="n">
         <v>45413</v>
       </c>
-      <c r="B234" s="2">
+      <c r="B234" s="5" t="n">
         <v>5.25</v>
       </c>
     </row>
-    <row r="235" spans="1:2">
-      <c r="A235" s="4">
+    <row r="235">
+      <c r="A235" s="6" t="n">
         <v>45444</v>
       </c>
-      <c r="B235" s="2">
+      <c r="B235" s="5" t="n">
         <v>5.13</v>
       </c>
     </row>
-    <row r="236" spans="1:2">
-      <c r="A236" s="4">
+    <row r="236">
+      <c r="A236" s="6" t="n">
         <v>45474</v>
       </c>
-      <c r="B236" s="2">
+      <c r="B236" s="5" t="n">
         <v>5.12</v>
       </c>
     </row>
-    <row r="237" spans="1:2">
-      <c r="A237" s="4">
+    <row r="237">
+      <c r="A237" s="6" t="n">
         <v>45505</v>
       </c>
-      <c r="B237" s="2">
+      <c r="B237" s="5" t="n">
         <v>4.87</v>
       </c>
     </row>
-    <row r="238" spans="1:2">
-      <c r="A238" s="4">
+    <row r="238">
+      <c r="A238" s="6" t="n">
         <v>45536</v>
       </c>
-      <c r="B238" s="2">
+      <c r="B238" s="5" t="n">
         <v>4.68</v>
       </c>
     </row>
-    <row r="239" spans="1:2">
-      <c r="A239" s="4">
+    <row r="239">
+      <c r="A239" s="6" t="n">
         <v>45566</v>
       </c>
-      <c r="B239" s="2">
+      <c r="B239" s="5" t="n">
         <v>4.95</v>
       </c>
     </row>
-    <row r="240" spans="1:2">
-      <c r="A240" s="4">
+    <row r="240">
+      <c r="A240" s="6" t="n">
         <v>45597</v>
       </c>
-      <c r="B240" s="2">
+      <c r="B240" s="5" t="n">
         <v>5.14</v>
       </c>
     </row>
-    <row r="241" spans="1:2">
-      <c r="A241" s="4">
+    <row r="241">
+      <c r="A241" s="6" t="n">
         <v>45627</v>
       </c>
-      <c r="B241" s="2">
+      <c r="B241" s="5" t="n">
         <v>5.2</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2">
-      <c r="A242" s="4">
-        <v>45658</v>
-      </c>
-      <c r="B242" s="2">
-        <v>5.46</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2">
-      <c r="A243" s="4">
-        <v>45689</v>
-      </c>
-      <c r="B243" s="2">
-        <v>5.32</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2">
-      <c r="A244" s="4">
-        <v>45717</v>
-      </c>
-      <c r="B244" s="2">
-        <v>5.29</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2">
-      <c r="A245" s="4">
-        <v>45748</v>
-      </c>
-      <c r="B245" s="2">
-        <v>5.45</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2">
-      <c r="A246" s="4">
-        <v>45778</v>
-      </c>
-      <c r="B246" s="2">
-        <v>5.54</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2">
-      <c r="A247" s="4">
-        <v>45809</v>
-      </c>
-      <c r="B247" s="2">
-        <v>5.46</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2">
-      <c r="A248" s="4">
-        <v>45839</v>
-      </c>
-      <c r="B248" s="2">
-        <v>5.45</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2">
-      <c r="A249" s="4">
-        <v>45870</v>
-      </c>
-      <c r="B249" s="2">
-        <v>5.35</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2">
-      <c r="A250" s="4">
-        <v>45901</v>
-      </c>
-      <c r="B250" s="2">
-        <v>5.21</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2">
-      <c r="A251" s="4">
-        <v>45931</v>
-      </c>
-      <c r="B251" s="2">
-        <v>5.13</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2">
-      <c r="A252" s="4">
-        <v>45962</v>
-      </c>
-      <c r="B252" s="2">
-        <v>5.26</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2">
-      <c r="A253" s="4">
-        <v>45992</v>
-      </c>
-      <c r="B253" s="2">
-        <v>5.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>